<commit_message>
fix the margin and the forexAvg in the excel
</commit_message>
<xml_diff>
--- a/ExcelService/ExcelService/PdfToExcel/wwwroot/files/forex.xlsx
+++ b/ExcelService/ExcelService/PdfToExcel/wwwroot/files/forex.xlsx
@@ -88,19 +88,19 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -512,17 +512,17 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>يورو</t>
+          <t>اليورو</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1.1785</v>
+        <v>1.171</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1.1784</v>
+        <v>1.1709</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.1786</v>
+        <v>1.1711</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
@@ -533,17 +533,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>جنيه إسترليني</t>
+          <t>الجنيه الاسترليني</t>
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1.3632</v>
+        <v>1.353</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>1.363</v>
+        <v>1.3529</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>1.3634</v>
+        <v>1.3531</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
@@ -554,17 +554,17 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ين ياباني</t>
+          <t>اليين الياباني</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>156.685</v>
+        <v>157.775</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>156.66</v>
+        <v>157.77</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>156.71</v>
+        <v>157.78</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -575,17 +575,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>يوان صيني</t>
+          <t>اليوان الصيني</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>6.8005</v>
+        <v>6.7906</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>6.8004</v>
+        <v>6.7902</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>6.8006</v>
+        <v>6.7909</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -596,17 +596,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>ليرة تركية</t>
+          <t>الليرة التركية</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45.3309</v>
+        <v>45.4173</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45.2574</v>
+        <v>45.4149</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45.4044</v>
+        <v>45.4196</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -617,17 +617,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>ريال سعودي</t>
+          <t>الريال السعودي</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3.7821</v>
+        <v>3.7523</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>3.7502</v>
+        <v>3.7522</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>3.8139</v>
+        <v>3.7524</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -638,7 +638,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>ريال قطري</t>
+          <t>الريال القطري الجديد</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -659,17 +659,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>درهم إماراتي</t>
+          <t>الدرهم الاماراتي</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>3.6731</v>
+        <v>3.6725</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>3.673</v>
+        <v>3.6715</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>3.6732</v>
+        <v>3.6735</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -680,17 +680,17 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>دينار كويتي</t>
+          <t>الدينار الكويتي / جديد</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.3077</v>
+        <v>0.3083</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.3072</v>
+        <v>0.3078</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.3082</v>
+        <v>0.3088</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -701,7 +701,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>دينار بحريني</t>
+          <t>الدينار البحريني</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
@@ -722,7 +722,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>ريال عماني</t>
+          <t>الريال العماني</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -743,7 +743,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>دينار أردني</t>
+          <t>الدينار الاردني</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
@@ -764,17 +764,17 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>جنيه مصري</t>
+          <t>الجنيه المصري</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>52.72</v>
+        <v>52.87</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>52.67</v>
+        <v>52.82</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>52.77</v>
+        <v>52.92</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -785,17 +785,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>فرنك سويسري</t>
+          <t>الفرنك السويسري</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0.7764</v>
+        <v>0.7817</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.7761</v>
+        <v>0.7816</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.7766999999999999</v>
+        <v>0.7818000000000001</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -806,17 +806,17 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>دولار كندي</t>
+          <t>الدولار الكندي</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.3677</v>
+        <v>1.37</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1.3671</v>
+        <v>1.3699</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1.3682</v>
+        <v>1.3701</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -827,17 +827,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>كرونة دانماركية</t>
+          <t>الكورون الدانمركي</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>6.3403</v>
+        <v>6.3802</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>6.3369</v>
+        <v>6.3782</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>6.3437</v>
+        <v>6.3822</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -848,17 +848,17 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>كرونة سويدية</t>
+          <t>الكورون السويدي</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>9.2164</v>
+        <v>9.3073</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>9.204499999999999</v>
+        <v>9.3043</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>9.228300000000001</v>
+        <v>9.3103</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -869,17 +869,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>كرونة نرويجية</t>
+          <t>الكورون النرويجي</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>9.2066</v>
+        <v>9.189</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>9.189500000000001</v>
+        <v>9.186</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>9.223699999999999</v>
+        <v>9.192</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -890,17 +890,17 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>دولار أسترالي</t>
+          <t>الدولار الاسترالي</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.7248</v>
+        <v>0.724</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.7242</v>
+        <v>0.7239</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.7252999999999999</v>
+        <v>0.7241</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -911,17 +911,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>دينار جزائري</t>
+          <t>الدينار الجزائري</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>132.26</v>
+        <v>132.4955</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>131.602</v>
+        <v>131.836</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>132.918</v>
+        <v>133.155</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -932,11 +932,11 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>جنيه سوداني</t>
+          <t>الجنيه السوداني/الجديد</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>600.5</v>
+        <v>600</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>598</v>
@@ -953,17 +953,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>دينار ليبي</t>
+          <t>الدينار الليبي</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>6.3227</v>
+        <v>6.3279</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>6.2972</v>
+        <v>6.3023</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>6.3482</v>
+        <v>6.3534</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -974,38 +974,38 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>درهم مغربي</t>
+          <t>الدرهم المغربي</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>9.1211</v>
+        <v>9.1656</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>9.109999999999999</v>
+        <v>9.1616</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>9.132099999999999</v>
+        <v>9.169600000000001</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>IQD/100</t>
+          <t>IQD</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>دينار عراقي/100</t>
+          <t>الدينار العراقي/المانة</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>13.1</v>
+        <v>13.1017</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>13.08</v>
+        <v>12.8461</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13.12</v>
+        <v>13.3572</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -1016,35 +1016,35 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>روبل روسي</t>
+          <t>الروبل الروسي</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>74.1365</v>
+        <v>73.5462</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>73.97669999999999</v>
+        <v>73.30459999999999</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>74.2963</v>
+        <v>73.7878</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>IRR/100</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>ريال إيراني/100</t>
+          <t>الريال الايراني/المانة</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
+        <v>13120</v>
+      </c>
+      <c r="D27" s="4" t="n">
         <v>13115</v>
-      </c>
-      <c r="D27" s="4" t="n">
-        <v>13105</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>13125</v>
@@ -1053,22 +1053,22 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>YER/100</t>
+          <t>YER</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>ريال يمني/100</t>
+          <t>الريال اليمني/المانة</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2.3863</v>
+        <v>2.3865</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>2.3835</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>2.389</v>
+        <v>2.3895</v>
       </c>
     </row>
   </sheetData>

</xml_diff>